<commit_message>
remove solutions, update program
</commit_message>
<xml_diff>
--- a/Teachers/Data/climate_change.xlsx
+++ b/Teachers/Data/climate_change.xlsx
@@ -2640,7 +2640,7 @@
         <v>208.8870555132515</v>
       </c>
       <c r="F62">
-        <v>75.76493109489857</v>
+        <v>75.76493109489859</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2859,10 +2859,10 @@
         <v>10</v>
       </c>
       <c r="E68">
-        <v>82.6241728198832</v>
+        <v>82.62417281988321</v>
       </c>
       <c r="F68">
-        <v>22.48308786126397</v>
+        <v>22.48308786126396</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         <v>5</v>
       </c>
       <c r="E69">
-        <v>40.40304637653821</v>
+        <v>40.40304637653822</v>
       </c>
       <c r="F69">
         <v>112.7391619883984</v>
@@ -3007,7 +3007,7 @@
         <v>8</v>
       </c>
       <c r="E72">
-        <v>59.57301013362323</v>
+        <v>59.57301013362324</v>
       </c>
       <c r="F72">
         <v>58.55029766169557</v>
@@ -3044,7 +3044,7 @@
         <v>2</v>
       </c>
       <c r="E73">
-        <v>466.3700429736073</v>
+        <v>466.3700429736072</v>
       </c>
       <c r="F73">
         <v>160.3942259425719</v>
@@ -3081,7 +3081,7 @@
         <v>2</v>
       </c>
       <c r="E74">
-        <v>62.48368545506489</v>
+        <v>62.48368545506488</v>
       </c>
       <c r="F74">
         <v>88.85334182223501</v>
@@ -3155,7 +3155,7 @@
         <v>3</v>
       </c>
       <c r="E76">
-        <v>420.6832005100088</v>
+        <v>420.6832005100087</v>
       </c>
       <c r="F76">
         <v>134.4202660391122</v>
@@ -3232,7 +3232,7 @@
         <v>252.6372574041501</v>
       </c>
       <c r="F78">
-        <v>105.2649135174043</v>
+        <v>105.2649135174044</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3306,7 +3306,7 @@
         <v>237.5590999434498</v>
       </c>
       <c r="F80">
-        <v>67.21464772476241</v>
+        <v>67.2146477247624</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3414,7 +3414,7 @@
         <v>5</v>
       </c>
       <c r="E83">
-        <v>102.0906500120714</v>
+        <v>102.0906500120713</v>
       </c>
       <c r="F83">
         <v>83.53181029917772</v>
@@ -3639,7 +3639,7 @@
         <v>169.8122181663735</v>
       </c>
       <c r="F89">
-        <v>140.2352681179362</v>
+        <v>140.2352681179361</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3861,7 +3861,7 @@
         <v>385.0758631483059</v>
       </c>
       <c r="F95">
-        <v>95.14089807665073</v>
+        <v>95.14089807665074</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3932,7 +3932,7 @@
         <v>5</v>
       </c>
       <c r="E97">
-        <v>294.9655716923788</v>
+        <v>294.9655716923789</v>
       </c>
       <c r="F97">
         <v>127.2424768947427</v>
@@ -3972,7 +3972,7 @@
         <v>335.7774045112239</v>
       </c>
       <c r="F98">
-        <v>42.9541652099915</v>
+        <v>42.95416520999149</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         <v>272.1361442205957</v>
       </c>
       <c r="F99">
-        <v>49.57583657677301</v>
+        <v>49.57583657677303</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -4043,10 +4043,10 @@
         <v>9</v>
       </c>
       <c r="E100">
-        <v>239.9323649042626</v>
+        <v>239.9323649042625</v>
       </c>
       <c r="F100">
-        <v>-9.462103566847389</v>
+        <v>-9.462103566847411</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -4080,10 +4080,10 @@
         <v>9</v>
       </c>
       <c r="E101">
-        <v>523.0289008657162</v>
+        <v>523.0289008657161</v>
       </c>
       <c r="F101">
-        <v>86.28772611407877</v>
+        <v>86.28772611407875</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -4157,7 +4157,7 @@
         <v>249.0504494452507</v>
       </c>
       <c r="F103">
-        <v>88.52912782542023</v>
+        <v>88.52912782542022</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -4265,7 +4265,7 @@
         <v>0</v>
       </c>
       <c r="E106">
-        <v>437.2867622604698</v>
+        <v>437.2867622604697</v>
       </c>
       <c r="F106">
         <v>108.8359001478059</v>
@@ -4376,7 +4376,7 @@
         <v>9</v>
       </c>
       <c r="E109">
-        <v>292.3047043659509</v>
+        <v>292.3047043659508</v>
       </c>
       <c r="F109">
         <v>76.32980016229156</v>
@@ -4450,7 +4450,7 @@
         <v>2</v>
       </c>
       <c r="E111">
-        <v>3.756900894183957</v>
+        <v>3.756900894183912</v>
       </c>
       <c r="F111">
         <v>121.9092171481705</v>
@@ -4561,7 +4561,7 @@
         <v>1</v>
       </c>
       <c r="E114">
-        <v>27.09090176375287</v>
+        <v>27.09090176375288</v>
       </c>
       <c r="F114">
         <v>167.8563519135061</v>
@@ -4601,7 +4601,7 @@
         <v>168.575033117699</v>
       </c>
       <c r="F115">
-        <v>70.38908133744445</v>
+        <v>70.38908133744444</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -4675,7 +4675,7 @@
         <v>345.230217754858</v>
       </c>
       <c r="F117">
-        <v>43.78408622768544</v>
+        <v>43.78408622768543</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -4749,7 +4749,7 @@
         <v>240.4793525716181</v>
       </c>
       <c r="F119">
-        <v>95.07777188223915</v>
+        <v>95.07777188223913</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -4783,7 +4783,7 @@
         <v>11</v>
       </c>
       <c r="E120">
-        <v>155.7546494398131</v>
+        <v>155.7546494398132</v>
       </c>
       <c r="F120">
         <v>117.3825030533753</v>

</xml_diff>